<commit_message>
datos: base consolidada con la plantilla de septiembre
Doce lotes, cinco mas que en agosto. Con el recalculo de la plantilla se
recuperan el tiempo de desarrollo y el alimento por dia, que llegaban vacios.

Proteina y lipidos (V10 y V11) siguen pendientes del analisis bromatologico,
asi que el modelo en uso no cambia: sigue marcado como entrenado con datos
simulados.
</commit_message>
<xml_diff>
--- a/entregables/base-datos-consolidada.xlsx
+++ b/entregables/base-datos-consolidada.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -496,7 +496,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Lotes consolidados: 7.</t>
+          <t>Lotes consolidados: 12.</t>
         </is>
       </c>
     </row>
@@ -570,10 +570,17 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Las variables que la plantilla calcula con fórmulas (tiempo de desarrollo, alimento por día, temperatura, humedad, densidad, supervivencia y longitud final) se recalculan desde las hojas de alimentación y seguimiento, para no depender del programa con que se guardó el archivo.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Variables a la espera de laboratorio: V10, V11.</t>
         </is>
@@ -590,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -817,13 +824,13 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.1176</v>
+        <v>0.1837</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>27.8667</v>
+        <v>29.2185</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>67.16670000000001</v>
+        <v>57.0741</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>12</v>
@@ -837,7 +844,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>34</v>
+        <v>98</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>170</v>
@@ -845,7 +852,7 @@
       <c r="K4" s="4" t="n"/>
       <c r="L4" s="4" t="n"/>
       <c r="M4" s="2" t="n">
-        <v>100</v>
+        <v>12.3529</v>
       </c>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
@@ -868,25 +875,27 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1.0769</v>
+        <v>0.5143</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>27.9667</v>
+        <v>29.3583</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>64</v>
+        <v>56.125</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="n">
+        <v>525.2101</v>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Familia Gryllidae (especie por confirmar)</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>25</v>
@@ -894,7 +903,7 @@
       <c r="K5" s="4" t="n"/>
       <c r="L5" s="4" t="n"/>
       <c r="M5" s="2" t="n">
-        <v>100</v>
+        <v>16</v>
       </c>
       <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="n"/>
@@ -903,7 +912,11 @@
           <t>Experimental</t>
         </is>
       </c>
-      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Grillos llegaron ya medianos</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -917,25 +930,27 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.7692</v>
+        <v>0.2714</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>27.9667</v>
+        <v>29.1231</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>64</v>
+        <v>56.1538</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="n">
+        <v>759.0133</v>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Familia Gryllidae (especie por confirmar)</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>40</v>
@@ -943,7 +958,7 @@
       <c r="K6" s="4" t="n"/>
       <c r="L6" s="4" t="n"/>
       <c r="M6" s="2" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
@@ -970,25 +985,27 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.2714</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>27.9667</v>
+        <v>29.3583</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>64</v>
+        <v>56.125</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="n">
+        <v>928.5714</v>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Familia Gryllidae (especie por confirmar)</t>
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>52</v>
@@ -996,7 +1013,7 @@
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n"/>
       <c r="M7" s="2" t="n">
-        <v>100</v>
+        <v>13.4615</v>
       </c>
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
@@ -1005,7 +1022,11 @@
           <t>Experimental</t>
         </is>
       </c>
-      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Grillos llegaron ya medianos</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1019,25 +1040,27 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>0.1667</v>
+        <v>0.0435</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>27.9667</v>
+        <v>29.3583</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>64</v>
+        <v>56.125</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="n">
+        <v>1963.6364</v>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Familia Gryllidae (especie por confirmar)</t>
         </is>
       </c>
       <c r="I8" s="2" t="n">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>54</v>
@@ -1045,7 +1068,7 @@
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="n"/>
       <c r="M8" s="2" t="n">
-        <v>100</v>
+        <v>9.2593</v>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
@@ -1055,6 +1078,231 @@
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>LOTE 8</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.0172</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>29.3583</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>57.9167</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>721.0626</v>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Familia Gryllidae (especie por confirmar)</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="4" t="n"/>
+      <c r="L9" s="4" t="n"/>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="n"/>
+      <c r="O9" s="2" t="n"/>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LOTE 9</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Familia Gryllidae (especie por confirmar)</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
+      <c r="M10" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>LOTE 10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n">
+        <v>24.6667</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>74.16670000000001</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Familia Gryllidae (especie por confirmar)</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K11" s="4" t="n"/>
+      <c r="L11" s="4" t="n"/>
+      <c r="M11" s="2" t="n">
+        <v>86.66670000000001</v>
+      </c>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="n"/>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LOTE 11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Familia Gryllidae (especie por confirmar)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
+      <c r="M12" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LOTE 12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Familia Gryllidae (especie por confirmar)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="4" t="n"/>
+      <c r="L13" s="4" t="n"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="n"/>
+      <c r="O13" s="2" t="n"/>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1720,10 +1968,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>1</v>
@@ -1746,17 +1994,17 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>1</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -1772,17 +2020,17 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>1</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -1798,17 +2046,17 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>1</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -1824,10 +2072,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E6" s="5" t="n">
         <v>1</v>
@@ -1850,13 +2098,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.4285714285714285</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1876,10 +2124,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>1</v>
@@ -1902,17 +2150,17 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>1</v>
+        <v>0.9166666666666666</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -1928,17 +2176,17 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -1957,7 +2205,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
@@ -1983,7 +2231,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>0</v>
@@ -2006,17 +2254,17 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>1</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -2035,10 +2283,10 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2061,7 +2309,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
datos: base consolidada con la plantilla definitiva de octubre (13 lotes)
</commit_message>
<xml_diff>
--- a/entregables/base-datos-consolidada.xlsx
+++ b/entregables/base-datos-consolidada.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Léame" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Datos" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Diccionario" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Completitud" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dietas" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Léame" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Diccionario" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Completitud" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dietas" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -489,14 +489,14 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Generado el 2026-10-19 a partir de la plantilla de recolección.</t>
+          <t>Generado el 2026-10-20 a partir de la plantilla de recolección.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Lotes consolidados: 12.</t>
+          <t>Lotes consolidados: 13.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -854,7 +854,9 @@
       <c r="M4" s="2" t="n">
         <v>12.3529</v>
       </c>
-      <c r="N4" s="2" t="n"/>
+      <c r="N4" s="2" t="n">
+        <v>9.51</v>
+      </c>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
@@ -905,7 +907,9 @@
       <c r="M5" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="N5" s="2" t="n"/>
+      <c r="N5" s="2" t="n">
+        <v>17.06</v>
+      </c>
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
@@ -960,7 +964,9 @@
       <c r="M6" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="2" t="n"/>
+      <c r="N6" s="2" t="n">
+        <v>16.86</v>
+      </c>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1021,9 @@
       <c r="M7" s="2" t="n">
         <v>13.4615</v>
       </c>
-      <c r="N7" s="2" t="n"/>
+      <c r="N7" s="2" t="n">
+        <v>16.54</v>
+      </c>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="inlineStr">
         <is>
@@ -1070,7 +1078,9 @@
       <c r="M8" s="2" t="n">
         <v>9.2593</v>
       </c>
-      <c r="N8" s="2" t="n"/>
+      <c r="N8" s="2" t="n">
+        <v>10.25</v>
+      </c>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
@@ -1091,33 +1101,33 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.0172</v>
+        <v>0.0115</v>
       </c>
       <c r="D9" s="2" t="n">
-        <v>29.3583</v>
+        <v>29.532</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>57.9167</v>
+        <v>57.48</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="G9" s="2" t="n">
-        <v>721.0626</v>
-      </c>
+      <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="inlineStr">
         <is>
           <t>Familia Gryllidae (especie por confirmar)</t>
         </is>
       </c>
       <c r="I9" s="2" t="n">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="J9" s="2" t="n"/>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="n"/>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
+      <c r="N9" s="2" t="n">
+        <v>9.01</v>
+      </c>
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
         <is>
@@ -1139,10 +1149,10 @@
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n">
-        <v>25</v>
+        <v>25.1</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>75</v>
+        <v>73.16670000000001</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>12</v>
@@ -1154,7 +1164,7 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>38</v>
@@ -1164,7 +1174,9 @@
       <c r="M10" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="N10" s="2" t="n"/>
+      <c r="N10" s="2" t="n">
+        <v>14.28</v>
+      </c>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
@@ -1201,7 +1213,7 @@
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>15</v>
@@ -1211,7 +1223,9 @@
       <c r="M11" s="2" t="n">
         <v>86.66670000000001</v>
       </c>
-      <c r="N11" s="2" t="n"/>
+      <c r="N11" s="2" t="n">
+        <v>12.15</v>
+      </c>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
@@ -1233,7 +1247,7 @@
       </c>
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n">
-        <v>24.7</v>
+        <v>24.7833</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>75.5</v>
@@ -1248,7 +1262,7 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>38</v>
@@ -1258,7 +1272,9 @@
       <c r="M12" s="2" t="n">
         <v>100</v>
       </c>
-      <c r="N12" s="2" t="n"/>
+      <c r="N12" s="2" t="n">
+        <v>14.06</v>
+      </c>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
@@ -1290,7 +1306,9 @@
           <t>Familia Gryllidae (especie por confirmar)</t>
         </is>
       </c>
-      <c r="I13" s="2" t="n"/>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="J13" s="2" t="n"/>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="n"/>
@@ -1303,6 +1321,41 @@
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>LOTE 13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Familia Gryllidae (especie por confirmar)</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="4" t="n"/>
+      <c r="L14" s="4" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="n"/>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Experimental</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1968,10 +2021,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" s="5" t="n">
         <v>1</v>
@@ -1997,10 +2050,10 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.6153846153846154</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -2023,10 +2076,10 @@
         <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -2049,10 +2102,10 @@
         <v>11</v>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -2075,14 +2128,14 @@
         <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>1</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Completa</t>
+          <t>Parcial</t>
         </is>
       </c>
     </row>
@@ -2098,13 +2151,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -2124,10 +2177,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>1</v>
@@ -2150,13 +2203,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>0.9166666666666666</v>
+        <v>0.9230769230769231</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -2179,10 +2232,10 @@
         <v>10</v>
       </c>
       <c r="D10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -2205,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
@@ -2231,7 +2284,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>0</v>
@@ -2257,10 +2310,10 @@
         <v>10</v>
       </c>
       <c r="D13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.8333333333333334</v>
+        <v>0.7692307692307693</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -2280,13 +2333,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D14" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>0.1666666666666667</v>
+        <v>0.8461538461538461</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -2309,7 +2362,7 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>0</v>

</xml_diff>